<commit_message>
feat: implement executive brief presentation generation services, UI components, and enterprise security audit reports
</commit_message>
<xml_diff>
--- a/FINAL_OPPORTUNITY_AUDIT.xlsx
+++ b/FINAL_OPPORTUNITY_AUDIT.xlsx
@@ -808,7 +808,7 @@
         <v>1. Gross Strategic Opportunity (All Levers)</v>
       </c>
       <c r="B2">
-        <v>323.27</v>
+        <v>173.12</v>
       </c>
       <c r="C2" t="str">
         <v>SUM_BASE_CASES</v>
@@ -864,7 +864,7 @@
         <v>5. Net Defensible Opportunity</v>
       </c>
       <c r="B6">
-        <v>243.75</v>
+        <v>93.6</v>
       </c>
       <c r="C6" t="str">
         <v>NET_REALIZABLE_SAVINGS_TARGET</v>

</xml_diff>